<commit_message>
docs(f004): complete resident-town design rebaseline v1
</commit_message>
<xml_diff>
--- a/PM/feature_progress.xlsx
+++ b/PM/feature_progress.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nine Dimensions" sheetId="1" r:id="R50706e46cfd04fdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="R3bad549b05264c93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Batch" sheetId="3" r:id="Rd22286be39ee47a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role Capacity" sheetId="4" r:id="R59200ac035e84ac2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Rules" sheetId="5" r:id="Rcf6b5fe7bfc844ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nine Dimensions" sheetId="1" r:id="R578a6f3a5a1b4e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="R1e36a3e36bb143b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Batch" sheetId="3" r:id="R8856619453844266"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role Capacity" sheetId="4" r:id="Rca258570248646f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Rules" sheetId="5" r:id="Rb7a8fac3ca804bdd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -966,7 +966,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H19" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>0.9</x:v>
       </x:c>
       <x:c r="I19" s="26" t="n">
         <x:v>0</x:v>
@@ -993,19 +993,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q19" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="R19" s="25" t="str">
-        <x:v>DESIGN REBASELINE / FIGMA PENDING</x:v>
+        <x:v>DESIGN PACKAGE COMPLETE / FIGMA BLOCKED</x:v>
       </x:c>
       <x:c r="S19" s="25" t="str">
         <x:v>Codex /root</x:v>
       </x:c>
       <x:c r="T19" s="25" t="str">
-        <x:v>Approve the 1x1 footprint catalog and create/read back editable Figma/FigJam UE and state frames</x:v>
+        <x:v>User reviews the V1.0 footprint catalog and recommended defaults; restore edit-capable Figma/FigJam write-readback before runtime authorization</x:v>
       </x:c>
       <x:c r="U19" s="25" t="str">
-        <x:v>BLOCKED: Figma UE attachment; user design review pending; runtime not authorized. Old F004-DISTRICT.1 is historical migration input and its lock is released.</x:v>
+        <x:v>A-H design rebaseline, UI/UX priority, visual contract and DOCX/PDF package complete for review. BLOCKED: Figma UE attachment (skyfire Starter seat=View; MCP transport failed; browser/Chrome control unavailable). Runtime not authorized; old F004-DISTRICT.1 remains historical migration input.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -1535,7 +1535,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f6ccdaf923d49ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ae0af8874ba4723"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1598,7 +1598,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac41a0d9dbd2407f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffb2da27ecb94299"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1701,7 +1701,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e88556aa0ec493c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf668ad9b9fd4ba2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1864,7 +1864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc46eed9aa25e4d36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f03550d67ff45bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1983,7 +1983,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41ca39b593384770"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65303f5fb6804d59"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: sync canonical F004 progress workbook
</commit_message>
<xml_diff>
--- a/PM/feature_progress.xlsx
+++ b/PM/feature_progress.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nine Dimensions" sheetId="1" r:id="R0833fb6036664c0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="R7ce8ef5363b646e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Batch" sheetId="3" r:id="Rbe2eedea2ed34fe9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role Capacity" sheetId="4" r:id="Re34680758ebe4a00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Rules" sheetId="5" r:id="Rcea2bcf352eb46f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nine Dimensions" sheetId="1" r:id="Rfb0777d58e4d47a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="R71b30e2231fb4a24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Batch" sheetId="3" r:id="Rc48fcd53994048eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role Capacity" sheetId="4" r:id="Ra1f951298cc64125"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Rules" sheetId="5" r:id="R51c29d1973d8468d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -951,7 +951,7 @@
         <x:v>Animal Resident Town Spatial &amp; Autonomy Foundation</x:v>
       </x:c>
       <x:c r="C19" s="25" t="str">
-        <x:v>Producer-approved resident-town rebaseline / Penpot editable handoff</x:v>
+        <x:v>Producer-approved resident-town rebaseline / verified Penpot editable handoff</x:v>
       </x:c>
       <x:c r="D19" s="25" t="str">
         <x:v>docs/features/F-004-resident-town-spatial-autonomy.md; output/penpot/F004-RESIDENT.1/README.md</x:v>
@@ -966,7 +966,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H19" s="26" t="n">
-        <x:v>0.95</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I19" s="26" t="n">
         <x:v>0</x:v>
@@ -993,19 +993,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q19" s="26" t="n">
-        <x:v>0.1055555556</x:v>
+        <x:v>0.1111111111111111</x:v>
       </x:c>
       <x:c r="R19" s="25" t="str">
-        <x:v>DESIGN PACKAGE V1.1 / PENPOT SOURCE PENDING</x:v>
+        <x:v>DESIGN PACKAGE V1.1 / PENPOT SOURCE VERIFIED / USER REVIEW PENDING</x:v>
       </x:c>
       <x:c r="S19" s="25" t="str">
         <x:v>Codex /root</x:v>
       </x:c>
       <x:c r="T19" s="25" t="str">
-        <x:v>Authenticate Penpot; import and read back 8 screens + 4 flows; user reviews V1.1 footprint catalog and recommended defaults</x:v>
+        <x:v>User reviews the 1x1 footprint catalog and recommended resident/offline/order defaults; approve the design baseline before any runtime slice</x:v>
       </x:c>
       <x:c r="U19" s="25" t="str">
-        <x:v>V1.1 formal design, UI/UX priority, visual contract, Penpot SVG import sources and static review previews complete. PENDING: authenticated Penpot editable-file import/readback and user design review. Runtime not authorized; F003 remains accepted baseline and old F004-DISTRICT.1 is historical migration input.</x:v>
+        <x:v>Authenticated Penpot file/import/reopen/object readback verified. PENDING: cloud export archive and user detailed design review. No file lock. Runtime not authorized; F003 remains baseline and old F004-DISTRICT.1 remains historical input.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -1535,7 +1535,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c3bb271e86e4245"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd38c944bac9f42b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1589,7 +1589,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D5" s="17" t="str">
-        <x:v>Authenticate Penpot, import/read back F004 V1.1 boards, then obtain user design review</x:v>
+        <x:v>Review F004 footprint catalog/defaults and Penpot package; runtime remains unauthorized</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1598,7 +1598,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2086389aa70d4920"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf552170e21a42c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1683,16 +1683,16 @@
         <x:v>Codex /root</x:v>
       </x:c>
       <x:c r="E5" s="17" t="str">
-        <x:v>PENPOT SOURCE PENDING</x:v>
+        <x:v>PENPOT READBACK VERIFIED / USER REVIEW PENDING</x:v>
       </x:c>
       <x:c r="F5" s="17" t="str">
-        <x:v>V1.1 formal design plus 8 screen boards, 4 flow boards, 14 readback objects and 720 x 1280 previews ready</x:v>
+        <x:v>Authenticated file, 8 screen groups, 4 flow groups, 14 object IDs and nested vector readback verified</x:v>
       </x:c>
       <x:c r="G5" s="17" t="str">
-        <x:v>Authenticated Penpot import/readback and user review of footprint catalog/defaults</x:v>
+        <x:v>User approves footprint catalog/defaults and visual/UI contract; then issue separate runtime-slice receipt</x:v>
       </x:c>
       <x:c r="H5" s="17" t="str">
-        <x:v>No project file lock. Penpot cloud authentication/readback pending; runtime_authority=false</x:v>
+        <x:v>No file lock. Cloud export archive and user detailed review pending; runtime_authority=false</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1701,7 +1701,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re34318de724f40c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R005e332f5ca94363"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1864,7 +1864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6487eaae33714783"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa7ebcbea6f6445e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1983,7 +1983,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a1670320a594820"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dc9c91cd49d46f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: ship F004 animal resident runtime slice
</commit_message>
<xml_diff>
--- a/PM/feature_progress.xlsx
+++ b/PM/feature_progress.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nine Dimensions" sheetId="1" r:id="Rfb0777d58e4d47a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="R71b30e2231fb4a24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Batch" sheetId="3" r:id="Rc48fcd53994048eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role Capacity" sheetId="4" r:id="Ra1f951298cc64125"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Rules" sheetId="5" r:id="R51c29d1973d8468d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nine Dimensions" sheetId="1" r:id="R267dd0d7311044fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="R12a735e534204094"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Batch" sheetId="3" r:id="R659edde245524d19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Role Capacity" sheetId="4" r:id="R87d891da52814002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update Rules" sheetId="5" r:id="R84fc8f880d254ec0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -648,16 +648,16 @@
         <x:v>Design doc</x:v>
       </x:c>
       <x:c r="B6" s="18" t="n">
-        <x:v>0.395</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="C6" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D6" s="17" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="E6" s="17" t="str">
-        <x:v>F-004 V1.1 is ready for Penpot import/review; F-005 to F-010 still need dedicated design sources</x:v>
+        <x:v>F-004 representative slice approved; F-005 to F-010 still need dedicated design sources</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -665,16 +665,16 @@
         <x:v>Numeric table</x:v>
       </x:c>
       <x:c r="B7" s="18" t="n">
-        <x:v>0.3</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="C7" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D7" s="17" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="E7" s="17" t="str">
-        <x:v>F-004 configuration tables wait for approved Penpot/design gate; F-005 to F-010 need original tables</x:v>
+        <x:v>F-004 seven runtime tables approved; F-005 to F-010 still need original configuration</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -682,16 +682,16 @@
         <x:v>Code</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
-        <x:v>0.3</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="C8" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D8" s="17" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="E8" s="17" t="str">
-        <x:v>Only F-001 to F-003 have runtime behavior; F-004 runtime is not authorized</x:v>
+        <x:v>F-004 native Godot loop approved; F-005 to F-010 remain roadmap-only</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -699,16 +699,16 @@
         <x:v>Scene</x:v>
       </x:c>
       <x:c r="B9" s="18" t="n">
-        <x:v>0.2222222222</x:v>
+        <x:v>0.3333333333</x:v>
       </x:c>
       <x:c r="C9" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D9" s="17" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="E9" s="17" t="str">
-        <x:v>F-004 scene rules are designed but not runtime; future scene decisions remain unsourced</x:v>
+        <x:v>F-004 representative scene approved; future scenes need separate feature gates</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -716,16 +716,16 @@
         <x:v>UI</x:v>
       </x:c>
       <x:c r="B10" s="18" t="n">
-        <x:v>0.3</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="C10" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D10" s="17" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="E10" s="17" t="str">
-        <x:v>F-004 UI/UE has Penpot import sources but no authenticated editable-file approval</x:v>
+        <x:v>F-004 native responsive UI approved; future screens remain unauthorised</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -733,16 +733,16 @@
         <x:v>Icon/image</x:v>
       </x:c>
       <x:c r="B11" s="18" t="n">
-        <x:v>0.2222222222</x:v>
+        <x:v>0.3333333333</x:v>
       </x:c>
       <x:c r="C11" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D11" s="17" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="E11" s="17" t="str">
-        <x:v>F-004 formal runtime art waits for design approval; future visual contracts remain unsourced</x:v>
+        <x:v>F-004 6+1 runtime asset set approved; future asset families need whole-set review</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -750,16 +750,16 @@
         <x:v>Scene integration</x:v>
       </x:c>
       <x:c r="B12" s="18" t="n">
-        <x:v>0.2222222222</x:v>
+        <x:v>0.3333333333</x:v>
       </x:c>
       <x:c r="C12" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D12" s="17" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="E12" s="17" t="str">
-        <x:v>F-004 representative runtime slice is not authorized; future scene integration remains unsourced</x:v>
+        <x:v>F-004 scene integration approved; no broad scale-out authority</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -767,16 +767,16 @@
         <x:v>Image integration</x:v>
       </x:c>
       <x:c r="B13" s="18" t="n">
-        <x:v>0.2222222222</x:v>
+        <x:v>0.3333333333</x:v>
       </x:c>
       <x:c r="C13" s="17" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D13" s="17" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="E13" s="17" t="str">
-        <x:v>F-004 runtime asset integration is not authorized; future image integration remains unsourced</x:v>
+        <x:v>F-004 approved assets integrated; future families remain separately gated</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -784,16 +784,16 @@
         <x:v>UI integration</x:v>
       </x:c>
       <x:c r="B14" s="18" t="n">
-        <x:v>0.3</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="C14" s="17" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D14" s="17" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="E14" s="17" t="str">
-        <x:v>F-004 has no runtime UI authority until Penpot readback and user review pass</x:v>
+        <x:v>F-004 runtime UI integration approved; Android/release validation remains separate</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -801,16 +801,16 @@
         <x:v>Feature total</x:v>
       </x:c>
       <x:c r="B15" s="22" t="n">
-        <x:v>0.3105555556</x:v>
+        <x:v>0.4</x:v>
       </x:c>
       <x:c r="C15" s="21" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D15" s="21" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="E15" s="21" t="str">
-        <x:v>F-004 is at design rebaseline review; F-005 to F-010 remain roadmap-only</x:v>
+        <x:v>F-004 representative slice complete; F-005 to F-010 remain roadmap-only</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -951,16 +951,16 @@
         <x:v>Animal Resident Town Spatial &amp; Autonomy Foundation</x:v>
       </x:c>
       <x:c r="C19" s="25" t="str">
-        <x:v>Producer-approved resident-town rebaseline / verified Penpot editable handoff</x:v>
+        <x:v>Producer-approved resident-town representative runtime slice / verified Penpot editable handoff</x:v>
       </x:c>
       <x:c r="D19" s="25" t="str">
-        <x:v>docs/features/F-004-resident-town-spatial-autonomy.md; output/penpot/F004-RESIDENT.1/README.md</x:v>
+        <x:v>docs/features/F-004-resident-town-spatial-autonomy.md; docs/evidence/F004-RESIDENT.1/README.md; output/penpot/F004-RESIDENT.1/README.md</x:v>
       </x:c>
       <x:c r="E19" s="25" t="str">
-        <x:v>Pending F004-RESIDENT.1 grid, resident, job, workplace, vehicle-order and locale schemas after Penpot design approval</x:v>
+        <x:v>config/tables/f004_resident_grid.csv; f004_resident_types.csv; f004_resident_jobs.csv; f004_resident_workplaces.csv; f004_vehicle_orders.csv; f004_vehicle_routes.csv; f004_resident_locale.csv</x:v>
       </x:c>
       <x:c r="F19" s="25" t="str">
-        <x:v>PD-002 + PD-003 / F004-RESIDENT.1 V1.1: visible animal residents walk roads, live, work, carry goods and fulfill world-vehicle orders; Penpot is the formal editable source</x:v>
+        <x:v>PD-002 + PD-003 / F004-RESIDENT.1 V1.2: visible residents autonomously work and fulfill a world-vehicle order; representative slice approved</x:v>
       </x:c>
       <x:c r="G19" s="25" t="str">
         <x:v>P0</x:v>
@@ -969,43 +969,43 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I19" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J19" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K19" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L19" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M19" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N19" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O19" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="P19" s="26" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Q19" s="26" t="n">
-        <x:v>0.1111111111111111</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="R19" s="25" t="str">
-        <x:v>DESIGN PACKAGE V1.1 / PENPOT SOURCE VERIFIED / USER REVIEW PENDING</x:v>
+        <x:v>RUNTIME_SLICE_APPROVED / SCALE_OUT_NOT_AUTHORIZED</x:v>
       </x:c>
       <x:c r="S19" s="25" t="str">
         <x:v>Codex /root</x:v>
       </x:c>
       <x:c r="T19" s="25" t="str">
-        <x:v>User reviews the 1x1 footprint catalog and recommended resident/offline/order defaults; approve the design baseline before any runtime slice</x:v>
+        <x:v>Producer may separately authorize one scale-out feature identity; F-005 remains roadmap-only</x:v>
       </x:c>
       <x:c r="U19" s="25" t="str">
-        <x:v>Authenticated Penpot file/import/reopen/object readback verified. PENDING: cloud export archive and user detailed design review. No file lock. Runtime not authorized; F003 remains baseline and old F004-DISTRICT.1 remains historical input.</x:v>
+        <x:v>None for the representative slice. Penpot cloud download is an archival limitation only; Android/release and broad scale-out are not authorized.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="62" customHeight="1">
@@ -1535,7 +1535,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd38c944bac9f42b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raee5a0e1f0df4862"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1580,16 +1580,16 @@
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B5" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C5" s="17" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D5" s="17" t="str">
-        <x:v>Review F004 footprint catalog/defaults and Penpot package; runtime remains unauthorized</x:v>
+        <x:v>Await producer authorization for the next feature identity; F-005 remains roadmap-only</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1598,7 +1598,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf552170e21a42c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ccbd2809aba4e11"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1671,28 +1671,28 @@
     </x:row>
     <x:row r="5" ht="84" customHeight="1">
       <x:c r="A5" s="17" t="str">
-        <x:v>P0</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
-        <x:v>Animal Resident Town Spatial &amp; Autonomy Foundation</x:v>
+        <x:v>No active write task</x:v>
       </x:c>
       <x:c r="C5" s="17" t="str">
-        <x:v>F004-RESIDENT.1-DESIGN</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="D5" s="17" t="str">
         <x:v>Codex /root</x:v>
       </x:c>
       <x:c r="E5" s="17" t="str">
-        <x:v>PENPOT READBACK VERIFIED / USER REVIEW PENDING</x:v>
+        <x:v>F004 RUNTIME SLICE CLOSED</x:v>
       </x:c>
       <x:c r="F5" s="17" t="str">
-        <x:v>Authenticated file, 8 screen groups, 4 flow groups, 14 object IDs and nested vector readback verified</x:v>
+        <x:v>Representative loop, assets, runtime evidence and regressions approved</x:v>
       </x:c>
       <x:c r="G5" s="17" t="str">
-        <x:v>User approves footprint catalog/defaults and visual/UI contract; then issue separate runtime-slice receipt</x:v>
+        <x:v>Create a new RAG/control-plane receipt only after a separate scale-out decision</x:v>
       </x:c>
       <x:c r="H5" s="17" t="str">
-        <x:v>No file lock. Cloud export archive and user detailed review pending; runtime_authority=false</x:v>
+        <x:v>None; Penpot cloud download is a non-blocking archival limitation</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1701,7 +1701,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R005e332f5ca94363"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5febe3b159b46c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1772,10 +1772,10 @@
         <x:v>Occupied</x:v>
       </x:c>
       <x:c r="E5" s="17" t="str">
-        <x:v>F-003 capture closure</x:v>
+        <x:v>Monitor accepted F004 slice</x:v>
       </x:c>
       <x:c r="F5" s="17" t="str">
-        <x:v>Keep one writer and verify reviewed visual evidence</x:v>
+        <x:v>Do not activate scale-out without a new feature source and receipt</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="35" customHeight="1">
@@ -1786,16 +1786,16 @@
         <x:v>design-owner</x:v>
       </x:c>
       <x:c r="C6" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="17" t="str">
-        <x:v>Occupied</x:v>
+        <x:v>Available</x:v>
       </x:c>
       <x:c r="E6" s="17" t="str">
-        <x:v>F-003 capture review</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="F6" s="17" t="str">
-        <x:v>Hold F-004/F-005 as roadmap only</x:v>
+        <x:v>F004 design and Penpot source closed for the representative slice</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="35" customHeight="1">
@@ -1806,16 +1806,16 @@
         <x:v>engineering-owner</x:v>
       </x:c>
       <x:c r="C7" s="17" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="17" t="str">
-        <x:v>Occupied</x:v>
+        <x:v>Available</x:v>
       </x:c>
       <x:c r="E7" s="17" t="str">
-        <x:v>F-003 visual capture</x:v>
+        <x:v>—</x:v>
       </x:c>
       <x:c r="F7" s="17" t="str">
-        <x:v>Keep runtime behavior stable during capture</x:v>
+        <x:v>F004 runtime write set returned</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="35" customHeight="1">
@@ -1823,7 +1823,7 @@
         <x:v>Art owner</x:v>
       </x:c>
       <x:c r="B8" s="17" t="str">
-        <x:v>—</x:v>
+        <x:v>art-owner</x:v>
       </x:c>
       <x:c r="C8" s="17" t="n">
         <x:v>0</x:v>
@@ -1835,7 +1835,7 @@
         <x:v>—</x:v>
       </x:c>
       <x:c r="F8" s="17" t="str">
-        <x:v>No separate art task; vector placeholders are approved</x:v>
+        <x:v>F004 representative asset set approved; no batch art task</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="35" customHeight="1">
@@ -1852,10 +1852,10 @@
         <x:v>Available</x:v>
       </x:c>
       <x:c r="E9" s="17" t="str">
-        <x:v>Matrix refresh after close</x:v>
+        <x:v>Final source/RAG/Git synchronization</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
-        <x:v>Keep normal checks quiet</x:v>
+        <x:v>Keep routine checks quiet after closure</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1864,7 +1864,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa7ebcbea6f6445e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17a8654ddac241a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1983,7 +1983,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dc9c91cd49d46f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae61994fa27946fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>